<commit_message>
Clarify how public files are served in deployment
</commit_message>
<xml_diff>
--- a/public/inbound-template.xlsx
+++ b/public/inbound-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\greyd\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{286C6F5B-8253-4D95-A0AD-129BB9AEDE2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6AF2DC4-8BA4-4CA0-9BE2-B95A6BD60FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DAB60061-D38D-4A2D-81C9-86013AA8F984}"/>
+    <workbookView xWindow="1836" yWindow="4896" windowWidth="17280" windowHeight="8880" xr2:uid="{DAB60061-D38D-4A2D-81C9-86013AA8F984}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,19 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>발송일</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>상품명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>옵션</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>재고수량</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -65,6 +53,14 @@
   </si>
   <si>
     <t>비고</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>상품명+옵션</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>신청날짜</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -438,33 +434,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{220BFE2D-9566-465A-8F53-A60801C8CBF4}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="2" max="2" width="19.09765625" customWidth="1"/>
+    <col min="6" max="6" width="18.09765625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>